<commit_message>
Revise pandas chapter data workflow
</commit_message>
<xml_diff>
--- a/新章节编辑/pandas/backup/data/company_full_summary.xlsx
+++ b/新章节编辑/pandas/backup/data/company_full_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="59">
   <si>
     <t>证券代码</t>
   </si>
@@ -40,24 +40,12 @@
     <t>000002</t>
   </si>
   <si>
-    <t>000001</t>
-  </si>
-  <si>
-    <t>600015</t>
-  </si>
-  <si>
-    <t>600016</t>
+    <t>000400</t>
   </si>
   <si>
     <t>000338</t>
   </si>
   <si>
-    <t>000538</t>
-  </si>
-  <si>
-    <t>000513</t>
-  </si>
-  <si>
     <t>000555</t>
   </si>
   <si>
@@ -67,28 +55,22 @@
     <t>000006</t>
   </si>
   <si>
-    <t>600000</t>
-  </si>
-  <si>
     <t>000049</t>
   </si>
   <si>
     <t>000153</t>
   </si>
   <si>
+    <t>000333</t>
+  </si>
+  <si>
     <t>000016</t>
   </si>
   <si>
-    <t>000333</t>
-  </si>
-  <si>
     <t>000020</t>
   </si>
   <si>
-    <t>000007</t>
-  </si>
-  <si>
-    <t>000158</t>
+    <t>000014</t>
   </si>
   <si>
     <t>000559</t>
@@ -100,16 +82,19 @@
     <t>000021</t>
   </si>
   <si>
-    <t>000521</t>
-  </si>
-  <si>
     <t>000070</t>
   </si>
   <si>
+    <t>000423</t>
+  </si>
+  <si>
     <t>000004</t>
   </si>
   <si>
-    <t>000423</t>
+    <t>000403</t>
+  </si>
+  <si>
+    <t>000682</t>
   </si>
   <si>
     <t>深纺织A</t>
@@ -124,24 +109,12 @@
     <t>万科A</t>
   </si>
   <si>
-    <t>平安银行</t>
-  </si>
-  <si>
-    <t>华夏银行</t>
-  </si>
-  <si>
-    <t>民生银行</t>
+    <t>许继电气</t>
   </si>
   <si>
     <t>潍柴动力</t>
   </si>
   <si>
-    <t>云南白药</t>
-  </si>
-  <si>
-    <t>丽珠集团</t>
-  </si>
-  <si>
     <t>神州信息</t>
   </si>
   <si>
@@ -151,49 +124,55 @@
     <t>深振业A</t>
   </si>
   <si>
-    <t>浦发银行</t>
-  </si>
-  <si>
     <t>德赛电池</t>
   </si>
   <si>
     <t>丰原药业</t>
   </si>
   <si>
+    <t>美的集团</t>
+  </si>
+  <si>
     <t>深康佳A</t>
   </si>
   <si>
-    <t>美的集团</t>
-  </si>
-  <si>
     <t>深华发A</t>
   </si>
   <si>
-    <t>*ST 全新</t>
-  </si>
-  <si>
-    <t>常山北明</t>
+    <t>沙河股份</t>
   </si>
   <si>
     <t>万向钱潮</t>
   </si>
   <si>
-    <t>*ST 万方</t>
+    <t>万方发展</t>
   </si>
   <si>
     <t>深科技</t>
   </si>
   <si>
-    <t>长虹美菱</t>
-  </si>
-  <si>
     <t>特发信息</t>
   </si>
   <si>
+    <t>东阿阿胶</t>
+  </si>
+  <si>
+    <t>国农科技</t>
+  </si>
+  <si>
     <t>国华网安</t>
   </si>
   <si>
-    <t>东阿阿胶</t>
+    <t>双林生物</t>
+  </si>
+  <si>
+    <t>振兴生化</t>
+  </si>
+  <si>
+    <t>派林生物</t>
+  </si>
+  <si>
+    <t>东方电子</t>
   </si>
   <si>
     <t>计算机、通信和其他电子设备制造业</t>
@@ -205,16 +184,13 @@
     <t>汽车制造业</t>
   </si>
   <si>
-    <t>货币金融服务</t>
+    <t>电气机械及器材制造业</t>
+  </si>
+  <si>
+    <t>软件和信息技术服务业</t>
   </si>
   <si>
     <t>医药制造业</t>
-  </si>
-  <si>
-    <t>软件和信息技术服务业</t>
-  </si>
-  <si>
-    <t>电气机械及器材制造业</t>
   </si>
 </sst>
 </file>
@@ -603,10 +579,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="D2">
         <v>12.72</v>
@@ -626,10 +602,10 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D3">
         <v>27.87</v>
@@ -649,10 +625,10 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="D4">
         <v>78.53</v>
@@ -672,10 +648,10 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D5">
         <v>2976.79</v>
@@ -695,22 +671,22 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="D6">
-        <v>1062.12</v>
+        <v>82.17</v>
       </c>
       <c r="E6">
-        <v>1268.14</v>
+        <v>101.56</v>
       </c>
       <c r="F6">
-        <v>1432.42</v>
+        <v>111.91</v>
       </c>
       <c r="G6">
-        <v>0.3486423379655785</v>
+        <v>0.3619325788000487</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -718,22 +694,22 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D7">
-        <v>694.03</v>
+        <v>1592.56</v>
       </c>
       <c r="E7">
-        <v>827.6900000000001</v>
+        <v>1743.61</v>
       </c>
       <c r="F7">
-        <v>927.17</v>
+        <v>1974.91</v>
       </c>
       <c r="G7">
-        <v>0.3359220782963273</v>
+        <v>0.240085145928568</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -741,22 +717,22 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D8">
-        <v>1288.93</v>
+        <v>90.77</v>
       </c>
       <c r="E8">
-        <v>1549.82</v>
+        <v>101.46</v>
       </c>
       <c r="F8">
-        <v>1667.77</v>
+        <v>106.86</v>
       </c>
       <c r="G8">
-        <v>0.2939182112294694</v>
+        <v>0.1772612096507657</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -764,22 +740,22 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="D9">
-        <v>1592.56</v>
+        <v>282.49</v>
       </c>
       <c r="E9">
-        <v>1743.61</v>
+        <v>291.74</v>
       </c>
       <c r="F9">
-        <v>1974.91</v>
+        <v>330.96</v>
       </c>
       <c r="G9">
-        <v>0.240085145928568</v>
+        <v>0.1715812949130942</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -787,22 +763,22 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="D10">
-        <v>267.08</v>
+        <v>25.12</v>
       </c>
       <c r="E10">
-        <v>296.65</v>
+        <v>37.31</v>
       </c>
       <c r="F10">
-        <v>327.43</v>
+        <v>29.35</v>
       </c>
       <c r="G10">
-        <v>0.2259622584993262</v>
+        <v>0.1683917197452229</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -810,22 +786,22 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D11">
-        <v>88.61</v>
+        <v>172.49</v>
       </c>
       <c r="E11">
-        <v>93.84999999999999</v>
+        <v>184.43</v>
       </c>
       <c r="F11">
-        <v>105.2</v>
+        <v>193.98</v>
       </c>
       <c r="G11">
-        <v>0.1872249181807923</v>
+        <v>0.1245869325758013</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -833,22 +809,22 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="D12">
-        <v>90.77</v>
+        <v>30.13</v>
       </c>
       <c r="E12">
-        <v>101.46</v>
+        <v>32.38</v>
       </c>
       <c r="F12">
-        <v>106.86</v>
+        <v>33.21</v>
       </c>
       <c r="G12">
-        <v>0.1772612096507657</v>
+        <v>0.1022236973116495</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -856,22 +832,22 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D13">
-        <v>282.49</v>
+        <v>2596.65</v>
       </c>
       <c r="E13">
-        <v>291.74</v>
+        <v>2782.16</v>
       </c>
       <c r="F13">
-        <v>330.96</v>
+        <v>2842.21</v>
       </c>
       <c r="G13">
-        <v>0.1715812949130942</v>
+        <v>0.09456800107831231</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -879,22 +855,22 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D14">
-        <v>25.12</v>
+        <v>461.27</v>
       </c>
       <c r="E14">
-        <v>37.31</v>
+        <v>551.1900000000001</v>
       </c>
       <c r="F14">
-        <v>29.35</v>
+        <v>503.52</v>
       </c>
       <c r="G14">
-        <v>0.1683917197452229</v>
+        <v>0.09159494439265514</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -902,22 +878,22 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D15">
-        <v>1542.58</v>
+        <v>6.37</v>
       </c>
       <c r="E15">
-        <v>1710.85</v>
+        <v>7.22</v>
       </c>
       <c r="F15">
-        <v>1746.87</v>
+        <v>6.92</v>
       </c>
       <c r="G15">
-        <v>0.1324339742509302</v>
+        <v>0.08634222919937207</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -925,22 +901,22 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="D16">
-        <v>172.49</v>
+        <v>3.58</v>
       </c>
       <c r="E16">
-        <v>184.43</v>
+        <v>4.38</v>
       </c>
       <c r="F16">
-        <v>193.98</v>
+        <v>3.47</v>
       </c>
       <c r="G16">
-        <v>0.1245869325758013</v>
+        <v>-0.03072625698324016</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -948,22 +924,22 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="D17">
-        <v>30.13</v>
+        <v>113.62</v>
       </c>
       <c r="E17">
-        <v>32.38</v>
+        <v>105.81</v>
       </c>
       <c r="F17">
-        <v>33.21</v>
+        <v>108.82</v>
       </c>
       <c r="G17">
-        <v>0.1022236973116495</v>
+        <v>-0.04224608343601488</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -971,22 +947,22 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D18">
-        <v>461.27</v>
+        <v>1.19</v>
       </c>
       <c r="E18">
-        <v>551.1900000000001</v>
+        <v>1.16</v>
       </c>
       <c r="F18">
-        <v>503.52</v>
+        <v>1.11</v>
       </c>
       <c r="G18">
-        <v>0.09159494439265514</v>
+        <v>-0.06722689075630239</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -994,22 +970,22 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="D19">
-        <v>2618.2</v>
+        <v>160.61</v>
       </c>
       <c r="E19">
-        <v>2793.81</v>
+        <v>132.24</v>
       </c>
       <c r="F19">
-        <v>2857.1</v>
+        <v>149.67</v>
       </c>
       <c r="G19">
-        <v>0.09124589412573525</v>
+        <v>-0.06811531037917951</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1017,22 +993,22 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D20">
-        <v>6.37</v>
+        <v>57.06</v>
       </c>
       <c r="E20">
-        <v>7.22</v>
+        <v>43.28</v>
       </c>
       <c r="F20">
-        <v>6.92</v>
+        <v>47.22</v>
       </c>
       <c r="G20">
-        <v>0.08634222919937207</v>
+        <v>-0.1724500525762356</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1040,22 +1016,22 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D21">
-        <v>0.42</v>
+        <v>73.38</v>
       </c>
       <c r="E21">
-        <v>0.42</v>
+        <v>29.59</v>
       </c>
       <c r="F21">
-        <v>0.45</v>
+        <v>34.09</v>
       </c>
       <c r="G21">
-        <v>0.0714285714285714</v>
+        <v>-0.5354319978195693</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1063,183 +1039,114 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C22" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="D22">
-        <v>96.56</v>
-      </c>
-      <c r="E22">
-        <v>94.47</v>
-      </c>
-      <c r="F22">
-        <v>98.84</v>
-      </c>
-      <c r="G22">
-        <v>0.02361226180613096</v>
+        <v>3.67</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C23" t="s">
-        <v>62</v>
-      </c>
-      <c r="D23">
-        <v>113.62</v>
+        <v>57</v>
       </c>
       <c r="E23">
-        <v>105.81</v>
-      </c>
-      <c r="F23">
-        <v>108.82</v>
-      </c>
-      <c r="G23">
-        <v>-0.04224608343601488</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C24" t="s">
-        <v>65</v>
-      </c>
-      <c r="D24">
-        <v>1.19</v>
-      </c>
-      <c r="E24">
-        <v>1.16</v>
+        <v>57</v>
       </c>
       <c r="F24">
-        <v>1.11</v>
-      </c>
-      <c r="G24">
-        <v>-0.06722689075630239</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C25" t="s">
-        <v>60</v>
-      </c>
-      <c r="D25">
-        <v>160.61</v>
+        <v>58</v>
       </c>
       <c r="E25">
-        <v>132.24</v>
-      </c>
-      <c r="F25">
-        <v>149.67</v>
-      </c>
-      <c r="G25">
-        <v>-0.06811531037917951</v>
+        <v>9.16</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C26" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="D26">
-        <v>174.9</v>
-      </c>
-      <c r="E26">
-        <v>165.53</v>
-      </c>
-      <c r="F26">
-        <v>153.88</v>
-      </c>
-      <c r="G26">
-        <v>-0.1201829616923957</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C27" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27">
-        <v>57.06</v>
-      </c>
-      <c r="E27">
-        <v>46.56</v>
+        <v>58</v>
       </c>
       <c r="F27">
-        <v>47.22</v>
-      </c>
-      <c r="G27">
-        <v>-0.1724500525762356</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C28" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="D28">
-        <v>3.67</v>
-      </c>
-      <c r="E28">
-        <v>1.08</v>
-      </c>
-      <c r="F28">
-        <v>2.81</v>
-      </c>
-      <c r="G28">
-        <v>-0.2343324250681199</v>
+        <v>30.42</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B29" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C29" t="s">
-        <v>64</v>
-      </c>
-      <c r="D29">
-        <v>73.38</v>
+        <v>57</v>
       </c>
       <c r="E29">
-        <v>29.59</v>
+        <v>34.19</v>
       </c>
       <c r="F29">
-        <v>34.09</v>
-      </c>
-      <c r="G29">
-        <v>-0.5354319978195693</v>
+        <v>37.19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>